<commit_message>
No watch band: a line is favourable or it is not
The amber rating is gone with the tolerance that defined it. rag() returns
Favourable, Unfavourable or No baseline; calc_rag_watch_at is removed from the
settings, the config CSV and the packs; the summary chips count two states;
the attention chips carry one shape; and the amber styling — the KPI and
country dots, the scorecard dots, the .rag.a badge, the attention chip and the
decision card's left rule — is deleted rather than left unreachable. What
needs attention is simply what is unfavourable.

calc_rag_green_at still sets where favourable starts, and is now the whole of
the policy.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/IWPB_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/IWPB_dashboard_config_pack.xlsx
@@ -4605,7 +4605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4706,22 +4706,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>calc_rag_watch_at</t>
+          <t>calc_rag_direction</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>calc_rag_direction</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>